<commit_message>
fix(pivots): reference generator — Excel-shaped slicer and timeline parts, valid pivot seeds (Task 2 fix round 1)
Mirror the Excel-written R1 template: ext URIs, defined names, slicer
cache tabular items, timeline cache state, AlternateContent and content
types; separate the source data from the pivot; independent seeded source
columns; bgColor for solid dxf fills; structural and determinism tests.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KTccUzeFqqMqTthqgFm9H
</commit_message>
<xml_diff>
--- a/tests/fixtures/xlsx-pivots/table-custom-dxf.xlsx
+++ b/tests/fixtures/xlsx-pivots/table-custom-dxf.xlsx
@@ -10,6 +10,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -43,9 +46,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -58,7 +62,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -121,7 +125,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>South</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -130,13 +134,13 @@
         </is>
       </c>
       <c r="C2">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="D2">
-        <v>6646</v>
+        <v>6799</v>
       </c>
       <c r="E2">
-        <v>54</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3">
@@ -151,19 +155,19 @@
         </is>
       </c>
       <c r="C3">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D3">
-        <v>4298.01</v>
+        <v>2066.01</v>
       </c>
       <c r="E3">
-        <v>38</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>West</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -172,13 +176,13 @@
         </is>
       </c>
       <c r="C4">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="D4">
-        <v>3942.02</v>
+        <v>1649.02</v>
       </c>
       <c r="E4">
-        <v>78</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5">
@@ -196,16 +200,16 @@
         <v>2023</v>
       </c>
       <c r="D5">
-        <v>2506.03</v>
+        <v>3500.03</v>
       </c>
       <c r="E5">
-        <v>16</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>West</t>
+          <t>South</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -214,13 +218,13 @@
         </is>
       </c>
       <c r="C6">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="D6">
-        <v>9070.04</v>
+        <v>7923.04</v>
       </c>
       <c r="E6">
-        <v>86</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>